<commit_message>
update phase 1 part 2
</commit_message>
<xml_diff>
--- a/files/BUS331_Investment_Committee_Decision_Record_Student.xlsx
+++ b/files/BUS331_Investment_Committee_Decision_Record_Student.xlsx
@@ -1798,10 +1798,10 @@
       </x:c>
       <x:c r="B5" s="53" t="str"/>
       <x:c r="C5" s="54" t="str">
-        <x:v>Own client discovery, the 12-month market view, IPS objectives and constraints, and the handoff from client needs to investment criteria.</x:v>
+        <x:v>Own client scenario analysis, the 12-month market view, IPS objectives and constraints, and the handoff from client needs to investment criteria.</x:v>
       </x:c>
       <x:c r="D5" s="54" t="str">
-        <x:v>Lead the client interview, document goals and RRTTLLU constraints, establish the macro context, and name unresolved information gaps.</x:v>
+        <x:v>Lead analysis of the assigned client scenarios, document goals and RRTTLLU constraints, establish the macro context, and label reasoned assumptions and information gaps.</x:v>
       </x:c>
       <x:c r="E5" s="54" t="str">
         <x:v>Test whether proposed allocations and securities fit the approved client mandate and the committee's market view.</x:v>
@@ -2162,7 +2162,7 @@
     </x:row>
     <x:row r="5" ht="30" customHeight="1">
       <x:c r="A5" s="37" t="str">
-        <x:v>Summarize AI output; do not paste transcripts. Unknown client information stays unknown. Do not enter real personal information or proprietary FactSet data into an AI tool.</x:v>
+        <x:v>Separate supplied case facts from labeled, reasoned assumptions. Mark unsupported exact values for confirmation. Summarize AI challenges; do not enter real personal information or proprietary FactSet data into an AI tool.</x:v>
       </x:c>
       <x:c r="B5" s="37"/>
       <x:c r="C5" s="37"/>

</xml_diff>